<commit_message>
lipit droplet starvation new experiments
</commit_message>
<xml_diff>
--- a/synuclein_inclusion_biogenesis_2024/image_analysis/lipid_droplet_mitochondria/102225_SUMMARY.xlsx
+++ b/synuclein_inclusion_biogenesis_2024/image_analysis/lipid_droplet_mitochondria/102225_SUMMARY.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,10 +466,20 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Total Lipid Droplet Surface Area</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Mitochondria Surface Area</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Average Distance between Lipid Droplets and Mitochondria</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Average Blue Density in Donut Lipid Droplets</t>
         </is>
@@ -500,9 +510,15 @@
         <v>207.1666666666667</v>
       </c>
       <c r="H2" t="n">
+        <v>1398</v>
+      </c>
+      <c r="I2" t="n">
+        <v>7427</v>
+      </c>
+      <c r="J2" t="n">
         <v>6.690018703409995</v>
       </c>
-      <c r="I2" t="n">
+      <c r="K2" t="n">
         <v>0.07114995665992488</v>
       </c>
     </row>
@@ -531,9 +547,15 @@
         <v>712.5</v>
       </c>
       <c r="H3" t="n">
+        <v>1971</v>
+      </c>
+      <c r="I3" t="n">
+        <v>9192</v>
+      </c>
+      <c r="J3" t="n">
         <v>10.47008210035245</v>
       </c>
-      <c r="I3" t="n">
+      <c r="K3" t="n">
         <v>0.07511482254697285</v>
       </c>
     </row>
@@ -562,9 +584,15 @@
         <v>390.5</v>
       </c>
       <c r="H4" t="n">
+        <v>1023</v>
+      </c>
+      <c r="I4" t="n">
+        <v>8348</v>
+      </c>
+      <c r="J4" t="n">
         <v>9.7182531580755</v>
       </c>
-      <c r="I4" t="n">
+      <c r="K4" t="n">
         <v>0.1105921912946012</v>
       </c>
     </row>
@@ -593,9 +621,15 @@
         <v>167.5</v>
       </c>
       <c r="H5" t="n">
+        <v>1508</v>
+      </c>
+      <c r="I5" t="n">
+        <v>10155</v>
+      </c>
+      <c r="J5" t="n">
         <v>8.915401733127092</v>
       </c>
-      <c r="I5" t="n">
+      <c r="K5" t="n">
         <v>0.09888521219520031</v>
       </c>
     </row>
@@ -624,9 +658,15 @@
         <v>236</v>
       </c>
       <c r="H6" t="n">
+        <v>1645</v>
+      </c>
+      <c r="I6" t="n">
+        <v>9891</v>
+      </c>
+      <c r="J6" t="n">
         <v>7.516844916112995</v>
       </c>
-      <c r="I6" t="n">
+      <c r="K6" t="n">
         <v>0.04431828587125721</v>
       </c>
     </row>
@@ -655,9 +695,15 @@
         <v>234.1666666666667</v>
       </c>
       <c r="H7" t="n">
+        <v>1541</v>
+      </c>
+      <c r="I7" t="n">
+        <v>7807</v>
+      </c>
+      <c r="J7" t="n">
         <v>5.8540312740106</v>
       </c>
-      <c r="I7" t="n">
+      <c r="K7" t="n">
         <v>0.1178593148185688</v>
       </c>
     </row>
@@ -686,9 +732,15 @@
         <v>583.25</v>
       </c>
       <c r="H8" t="n">
+        <v>3156</v>
+      </c>
+      <c r="I8" t="n">
+        <v>9261</v>
+      </c>
+      <c r="J8" t="n">
         <v>7.000925641245168</v>
       </c>
-      <c r="I8" t="n">
+      <c r="K8" t="n">
         <v>0.06192748940206919</v>
       </c>
     </row>
@@ -717,9 +769,15 @@
         <v>499.1428571428572</v>
       </c>
       <c r="H9" t="n">
+        <v>3747</v>
+      </c>
+      <c r="I9" t="n">
+        <v>7361</v>
+      </c>
+      <c r="J9" t="n">
         <v>1.362489806311421</v>
       </c>
-      <c r="I9" t="n">
+      <c r="K9" t="n">
         <v>0.1797199270724233</v>
       </c>
     </row>
@@ -748,9 +806,15 @@
         <v>460</v>
       </c>
       <c r="H10" t="n">
+        <v>2498</v>
+      </c>
+      <c r="I10" t="n">
+        <v>9041</v>
+      </c>
+      <c r="J10" t="n">
         <v>7.916012629240374</v>
       </c>
-      <c r="I10" t="n">
+      <c r="K10" t="n">
         <v>0.1260279109634908</v>
       </c>
     </row>
@@ -779,9 +843,15 @@
         <v>656</v>
       </c>
       <c r="H11" t="n">
+        <v>4368</v>
+      </c>
+      <c r="I11" t="n">
+        <v>7125</v>
+      </c>
+      <c r="J11" t="n">
         <v>7.966280288717754</v>
       </c>
-      <c r="I11" t="n">
+      <c r="K11" t="n">
         <v>0.1051787541128653</v>
       </c>
     </row>
@@ -810,9 +880,15 @@
         <v>742.5</v>
       </c>
       <c r="H12" t="n">
+        <v>5181</v>
+      </c>
+      <c r="I12" t="n">
+        <v>5319</v>
+      </c>
+      <c r="J12" t="n">
         <v>5.285557445739255</v>
       </c>
-      <c r="I12" t="n">
+      <c r="K12" t="n">
         <v>0.105050505050505</v>
       </c>
     </row>
@@ -841,9 +917,15 @@
         <v>542.3333333333334</v>
       </c>
       <c r="H13" t="n">
+        <v>3962</v>
+      </c>
+      <c r="I13" t="n">
+        <v>8107</v>
+      </c>
+      <c r="J13" t="n">
         <v>7.658296440609549</v>
       </c>
-      <c r="I13" t="n">
+      <c r="K13" t="n">
         <v>0.08719542015477115</v>
       </c>
     </row>
@@ -872,9 +954,15 @@
         <v>382</v>
       </c>
       <c r="H14" t="n">
+        <v>909</v>
+      </c>
+      <c r="I14" t="n">
+        <v>7964</v>
+      </c>
+      <c r="J14" t="n">
         <v>12.42161940611421</v>
       </c>
-      <c r="I14" t="n">
+      <c r="K14" t="n">
         <v>0.06040113288249234</v>
       </c>
     </row>
@@ -903,9 +991,15 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
+        <v>1216</v>
+      </c>
+      <c r="I15" t="n">
+        <v>5217</v>
+      </c>
+      <c r="J15" t="n">
         <v>2.980487123603726</v>
       </c>
-      <c r="I15" t="n">
+      <c r="K15" t="n">
         <v>0.1238563287499346</v>
       </c>
     </row>
@@ -934,9 +1028,15 @@
         <v>330.5</v>
       </c>
       <c r="H16" t="n">
+        <v>3196</v>
+      </c>
+      <c r="I16" t="n">
+        <v>6127</v>
+      </c>
+      <c r="J16" t="n">
         <v>3.984135471488256</v>
       </c>
-      <c r="I16" t="n">
+      <c r="K16" t="n">
         <v>0.1027780142447717</v>
       </c>
     </row>
@@ -965,9 +1065,15 @@
         <v>232</v>
       </c>
       <c r="H17" t="n">
+        <v>2818</v>
+      </c>
+      <c r="I17" t="n">
+        <v>6730</v>
+      </c>
+      <c r="J17" t="n">
         <v>7.214156998550304</v>
       </c>
-      <c r="I17" t="n">
+      <c r="K17" t="n">
         <v>0.0446306875851869</v>
       </c>
     </row>

</xml_diff>